<commit_message>
Add phase-aware Penka scoring and prediction workflow
</commit_message>
<xml_diff>
--- a/outputs/final_match_recommendations.xlsx
+++ b/outputs/final_match_recommendations.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K73"/>
+  <dimension ref="A1:M73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,27 +449,37 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>safe_expected_points</t>
+          <t>expected_penka_points</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>selected_by</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>favorite_1_0_prediction</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>recommended_strategy</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>recommended_prediction</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>recommendation_reason</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>refresh_required_before_match</t>
         </is>
       </c>
     </row>
@@ -499,27 +509,35 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>2.215721273276185</v>
+        <v>1.755523154987879</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -548,27 +566,35 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1.904253953335298</v>
+        <v>1.426576945768382</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -597,27 +623,35 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1.716202069273567</v>
+        <v>1.367106546836943</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -646,27 +680,35 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1.637122475313113</v>
+        <v>1.278456271271067</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -695,27 +737,35 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1.933790737042726</v>
+        <v>1.488558882005448</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -744,27 +794,35 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1.827076691866781</v>
+        <v>1.440024467192536</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M7" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -793,27 +851,35 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>2.564389982001048</v>
+        <v>1.938696838173352</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -842,27 +908,35 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>2.080652247097085</v>
+        <v>1.562760746097457</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M9" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -891,27 +965,35 @@
         </is>
       </c>
       <c r="G10" t="n">
-        <v>2.506118537629934</v>
+        <v>1.884991998197628</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M10" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -940,27 +1022,35 @@
         </is>
       </c>
       <c r="G11" t="n">
-        <v>1.696604963268674</v>
+        <v>1.333473473571547</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M11" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -989,27 +1079,35 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1.957338770631323</v>
+        <v>1.508673411484225</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M12" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1038,27 +1136,35 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>1.827076691866781</v>
+        <v>1.436321376152665</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1087,27 +1193,35 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1.827076691866781</v>
+        <v>1.435091775255023</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M14" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1136,27 +1250,35 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>1.858199610817391</v>
+        <v>1.484606184531527</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M15" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1185,27 +1307,35 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>1.649615379136533</v>
+        <v>1.334636557524165</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M16" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1234,27 +1364,35 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2.827024215120805</v>
+        <v>2.040973632929036</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M17" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1283,27 +1421,35 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>1.797126536522974</v>
+        <v>1.434862138330515</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M18" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1332,27 +1478,35 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>2.510521124286686</v>
+        <v>1.880591810490479</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M19" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1381,27 +1535,35 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>2.172796695272277</v>
+        <v>1.66268866317801</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M20" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -1430,27 +1592,35 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>1.413518007285681</v>
+        <v>1.151694573074271</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M21" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -1479,27 +1649,35 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>1.797126536522974</v>
+        <v>1.355562652081752</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M22" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -1528,27 +1706,35 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>1.957338770631323</v>
+        <v>1.507233995347682</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M23" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -1577,27 +1763,35 @@
         </is>
       </c>
       <c r="G24" t="n">
-        <v>1.462177753856218</v>
+        <v>1.191268753274762</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M24" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -1626,27 +1820,35 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>1.616235226403198</v>
+        <v>1.324863340276165</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M25" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -1675,27 +1877,35 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>2.827024215120805</v>
+        <v>2.070188709959749</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M26" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -1724,27 +1934,35 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>1.797126536522974</v>
+        <v>1.375110356238002</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M27" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -1773,27 +1991,35 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>2.048012460865912</v>
+        <v>1.613252347281032</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M28" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -1822,27 +2048,35 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>2.403816944250616</v>
+        <v>1.83252659983782</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M29" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -1871,27 +2105,35 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>1.65687498081312</v>
+        <v>1.310208104482419</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M30" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -1920,27 +2162,35 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>1.54910815594259</v>
+        <v>1.256396103229011</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M31" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -1969,27 +2219,35 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>1.76793384283286</v>
+        <v>1.379397353026854</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M32" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -2018,27 +2276,35 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>1.797126536522974</v>
+        <v>1.360571954886604</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M33" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -2067,27 +2333,35 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>2.005079142490461</v>
+        <v>1.604275777383214</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M34" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -2116,27 +2390,35 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>1.637122475313113</v>
+        <v>1.288510216502371</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M35" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -2165,27 +2447,35 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>1.904253953335298</v>
+        <v>1.446206833015282</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M36" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -2214,27 +2504,35 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>1.957338770631323</v>
+        <v>1.438399763824657</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M37" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -2263,27 +2561,35 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>2.378738905210191</v>
+        <v>1.766557675508336</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M38" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -2312,27 +2618,35 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>2.580964133397466</v>
+        <v>1.926955970533285</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M39" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -2361,27 +2675,35 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>1.933790737042726</v>
+        <v>1.503564699589998</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M40" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -2410,27 +2732,35 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>1.904253953335298</v>
+        <v>1.452550146186702</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M41" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -2459,27 +2789,35 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>1.54910815594259</v>
+        <v>1.216938050581892</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M42" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -2508,27 +2846,35 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>2.259463312356315</v>
+        <v>1.705304247725093</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M43" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -2557,27 +2903,35 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>2.872048456425783</v>
+        <v>2.106515517903942</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M44" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -2606,27 +2960,35 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>2.000700075692301</v>
+        <v>1.574626852272859</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M45" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -2655,27 +3017,35 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>2.474116345489455</v>
+        <v>1.834430508303675</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M46" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -2704,27 +3074,35 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>2.721659613675571</v>
+        <v>1.988387677367542</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M47" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -2753,27 +3131,35 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>1.608352162209543</v>
+        <v>1.309808122731809</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M48" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -2802,27 +3188,35 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>1.650226951207215</v>
+        <v>1.293572565310059</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M49" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -2851,27 +3245,35 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>2.234108835864963</v>
+        <v>1.64269242382841</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M50" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -2900,27 +3302,35 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>1.49056490207263</v>
+        <v>1.169824749476202</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M51" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -2949,27 +3359,35 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>2.501447783181691</v>
+        <v>1.843666016623124</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M52" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -2998,27 +3416,35 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>1.716202069273567</v>
+        <v>1.343761831922728</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M53" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -3047,27 +3473,35 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>1.904253953335298</v>
+        <v>1.437557684916533</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M54" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -3096,27 +3530,35 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>2.029716656759752</v>
+        <v>1.620560396487116</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M55" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -3145,27 +3587,35 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>2.234597296524142</v>
+        <v>1.726138684981324</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M56" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -3194,27 +3644,35 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>2.259463312356316</v>
+        <v>1.721394236376541</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M57" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -3243,27 +3701,35 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>2.048012460865912</v>
+        <v>1.643676208528625</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M58" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -3292,27 +3758,35 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>1.396213730119169</v>
+        <v>1.200560601383485</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M59" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="60">
@@ -3341,27 +3815,35 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>1.52749790669522</v>
+        <v>1.191770119371739</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M60" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -3390,27 +3872,35 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>2.15980406089399</v>
+        <v>1.612445764889097</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M61" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="62">
@@ -3439,27 +3929,35 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>2.658448083460662</v>
+        <v>1.971485874937763</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M62" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="63">
@@ -3488,27 +3986,35 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>1.904253953335298</v>
+        <v>1.43836616107441</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M63" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -3537,27 +4043,35 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>2.417755659238703</v>
+        <v>1.805810168560636</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M64" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="65">
@@ -3586,27 +4100,35 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>2.680641796319106</v>
+        <v>1.978060430256195</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M65" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -3631,31 +4153,39 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="G66" t="n">
-        <v>1.55000556677361</v>
+        <v>1.159615904779568</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M66" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="67">
@@ -3684,27 +4214,35 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>1.608352162209543</v>
+        <v>1.29608938918287</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M67" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="68">
@@ -3733,27 +4271,35 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>1.629115079523578</v>
+        <v>1.273676097048265</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M68" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -3782,27 +4328,35 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>1.858199610817391</v>
+        <v>1.473346311865261</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M69" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -3831,27 +4385,35 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>2.658448083460662</v>
+        <v>1.976533958651127</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M70" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -3880,27 +4442,35 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>1.608352162209543</v>
+        <v>1.29116849037689</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M71" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -3929,27 +4499,35 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>1.904253953335298</v>
+        <v>1.460372061208811</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>max_ev</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M72" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -3974,31 +4552,39 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="G73" t="n">
-        <v>2.526603006135452</v>
+        <v>1.841382504993279</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>exact_score_tiebreak</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>favorite_1_0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>penka_group_expected_value_refreshable</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>favorite_1_0 remains the historical default until a calibrated strategy beats it overall.</t>
-        </is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Real group-phase Penka EV with exact-score tie-breaking. Refresh close to kickoff; the earlier favorite_1_0 conclusion used an invalid points formula.</t>
+        </is>
+      </c>
+      <c r="M73" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>